<commit_message>
feat: PPM dinâmico por categoria e correções de sincronização v4
</commit_message>
<xml_diff>
--- a/app/development/catalogo/data/catalogo_codigos.xlsx
+++ b/app/development/catalogo/data/catalogo_codigos.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2118" uniqueCount="909">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2121" uniqueCount="911">
   <si>
     <t xml:space="preserve">CÓDIGO</t>
   </si>
@@ -2747,6 +2747,12 @@
   </si>
   <si>
     <t xml:space="preserve">PCI DISPLAY CM-550-L - IM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7041-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAIXA AMPLIFICADA CM-300-N BIV.</t>
   </si>
 </sst>
 </file>
@@ -2875,7 +2881,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C706"/>
+  <dimension ref="A1:C707"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.15"/>
@@ -10650,6 +10656,17 @@
         <v>5</v>
       </c>
     </row>
+    <row r="707" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A707" s="1" t="s">
+        <v>909</v>
+      </c>
+      <c r="B707" s="1" t="s">
+        <v>910</v>
+      </c>
+      <c r="C707" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>